<commit_message>
updated trim and fill code
</commit_message>
<xml_diff>
--- a/Plots/trim_fill_comparison_table.xlsx
+++ b/Plots/trim_fill_comparison_table.xlsx
@@ -47,49 +47,49 @@
     <t xml:space="preserve">unadj</t>
   </si>
   <si>
-    <t xml:space="preserve">1.34 (1.12-1.61)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.20 (0.97-1.49)</t>
+    <t xml:space="preserve">1.32 (1.16-1.50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.17 (1.02-1.33)</t>
   </si>
   <si>
     <t xml:space="preserve">adj</t>
   </si>
   <si>
-    <t xml:space="preserve">1.52 (1.24-1.86)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.36 (1.03-1.79)</t>
+    <t xml:space="preserve">1.60 (1.33-1.92)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.38 (1.11-1.71)</t>
   </si>
   <si>
     <t xml:space="preserve">best</t>
   </si>
   <si>
-    <t xml:space="preserve">1.34 (1.14-1.58)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.23 (1.02-1.49)</t>
+    <t xml:space="preserve">1.31 (1.16-1.48)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.16 (1.03-1.32)</t>
   </si>
   <si>
     <t xml:space="preserve">Ever</t>
   </si>
   <si>
-    <t xml:space="preserve">1.39 (1.23-1.58)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.34 (1.18-1.52)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.47 (1.27-1.71)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.36 (1.16-1.60)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.31 (1.19-1.44)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.25 (1.13-1.38)</t>
+    <t xml:space="preserve">1.42 (1.27-1.59)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.44 (1.30-1.60)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.51 (1.31-1.74)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.35 (1.26-1.44)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.35 (1.23-1.48)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.33 (1.24-1.43)</t>
   </si>
   <si>
     <t xml:space="preserve">By violence type</t>
@@ -619,7 +619,7 @@
         <v>12</v>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -642,7 +642,7 @@
         <v>15</v>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -665,7 +665,7 @@
         <v>18</v>
       </c>
       <c r="G6" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -688,7 +688,7 @@
         <v>21</v>
       </c>
       <c r="G7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -711,7 +711,7 @@
         <v>23</v>
       </c>
       <c r="G8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -734,145 +734,145 @@
         <v>25</v>
       </c>
       <c r="G9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="G10" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="D11" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E11" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="F11" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="D12" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E12" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F12" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="G12" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="D13" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E13" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="F13" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="G13" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="D14" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E14" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="F14" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="G14" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="C15" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="D15" t="s">
         <v>16</v>
       </c>
       <c r="E15" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="F15" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="G15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -880,7 +880,7 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="C16" t="s">
         <v>28</v>
@@ -889,13 +889,13 @@
         <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="F16" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="G16" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
@@ -903,7 +903,7 @@
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="C17" t="s">
         <v>31</v>
@@ -912,13 +912,13 @@
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="F17" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="G17" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -926,7 +926,7 @@
         <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="C18" t="s">
         <v>28</v>
@@ -935,10 +935,10 @@
         <v>13</v>
       </c>
       <c r="E18" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="F18" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="G18" t="n">
         <v>3</v>
@@ -949,7 +949,7 @@
         <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="C19" t="s">
         <v>31</v>
@@ -958,13 +958,13 @@
         <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="F19" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="G19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -972,7 +972,7 @@
         <v>26</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="C20" t="s">
         <v>28</v>
@@ -981,13 +981,13 @@
         <v>16</v>
       </c>
       <c r="E20" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="F20" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="G20" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -995,7 +995,7 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="C21" t="s">
         <v>31</v>
@@ -1004,13 +1004,13 @@
         <v>16</v>
       </c>
       <c r="E21" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="F21" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="G21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -1018,7 +1018,7 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="C22" t="s">
         <v>28</v>
@@ -1027,13 +1027,13 @@
         <v>10</v>
       </c>
       <c r="E22" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="F22" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="G22" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23">
@@ -1041,7 +1041,7 @@
         <v>26</v>
       </c>
       <c r="B23" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="C23" t="s">
         <v>31</v>
@@ -1050,13 +1050,13 @@
         <v>10</v>
       </c>
       <c r="E23" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="F23" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="G23" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24">
@@ -1064,7 +1064,7 @@
         <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="C24" t="s">
         <v>28</v>
@@ -1073,13 +1073,13 @@
         <v>13</v>
       </c>
       <c r="E24" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="F24" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="G24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -1087,7 +1087,7 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="C25" t="s">
         <v>31</v>
@@ -1096,13 +1096,13 @@
         <v>13</v>
       </c>
       <c r="E25" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="F25" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
@@ -1110,7 +1110,7 @@
         <v>26</v>
       </c>
       <c r="B26" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="C26" t="s">
         <v>28</v>
@@ -1119,13 +1119,13 @@
         <v>16</v>
       </c>
       <c r="E26" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="F26" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="G26" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27">
@@ -1133,7 +1133,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="C27" t="s">
         <v>31</v>
@@ -1142,13 +1142,13 @@
         <v>16</v>
       </c>
       <c r="E27" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="F27" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="G27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28">
@@ -1156,7 +1156,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="C28" t="s">
         <v>28</v>
@@ -1165,12 +1165,150 @@
         <v>10</v>
       </c>
       <c r="E28" t="s">
+        <v>56</v>
+      </c>
+      <c r="F28" t="s">
+        <v>57</v>
+      </c>
+      <c r="G28" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" t="s">
+        <v>31</v>
+      </c>
+      <c r="D29" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" t="s">
+        <v>58</v>
+      </c>
+      <c r="F29" t="s">
+        <v>59</v>
+      </c>
+      <c r="G29" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>26</v>
+      </c>
+      <c r="B30" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" t="s">
+        <v>28</v>
+      </c>
+      <c r="D30" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30" t="s">
+        <v>60</v>
+      </c>
+      <c r="F30" t="s">
+        <v>61</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" t="s">
+        <v>31</v>
+      </c>
+      <c r="D31" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" t="s">
+        <v>62</v>
+      </c>
+      <c r="F31" t="s">
+        <v>63</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>26</v>
+      </c>
+      <c r="B32" t="s">
+        <v>55</v>
+      </c>
+      <c r="C32" t="s">
+        <v>28</v>
+      </c>
+      <c r="D32" t="s">
+        <v>16</v>
+      </c>
+      <c r="E32" t="s">
+        <v>64</v>
+      </c>
+      <c r="F32" t="s">
+        <v>65</v>
+      </c>
+      <c r="G32" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>26</v>
+      </c>
+      <c r="B33" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" t="s">
+        <v>31</v>
+      </c>
+      <c r="D33" t="s">
+        <v>16</v>
+      </c>
+      <c r="E33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F33" t="s">
+        <v>67</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>26</v>
+      </c>
+      <c r="B34" t="s">
+        <v>68</v>
+      </c>
+      <c r="C34" t="s">
+        <v>28</v>
+      </c>
+      <c r="D34" t="s">
+        <v>10</v>
+      </c>
+      <c r="E34" t="s">
         <v>69</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F34" t="s">
         <v>70</v>
       </c>
-      <c r="G28" t="n">
+      <c r="G34" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>